<commit_message>
Api creation for single pdf text and Markes genration
</commit_message>
<xml_diff>
--- a/data/Final_markes.xlsx
+++ b/data/Final_markes.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -448,8 +448,33 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2/10
-Poor grammar and structure.</t>
+          <t>4/10
+Insufficient detail and poor structure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>assignment_CTV2_text</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>5/10
+Some understanding shown, but lacks depth and clarity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ayushResume_text</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>My apologies.  I am an AI and do not process images.  I was responding based on the assumption that you had provided handwritten answers previously.  Please provide the typed answers so I can evaluate them.</t>
         </is>
       </c>
     </row>

</xml_diff>